<commit_message>
Keep dynamic array formulas and switched-off error checks
openpyxl drops the cm attribute of cells and xl/metadata.xml, so dynamic
array formulas (FILTER, SORT, UNIQUE...) came back as legacy {=...}
arrays. The metadata part is exported as data/metadata.xml and cm is kept
on the cell record; both are written back on import. Metadata that also
describes values (pictures in cells) is still left out with a warning.

<ignoredErrors> is kept per sheet as XML; it was lost silently before.

Elements are inserted among the sheet's top-level elements only
(xmlfrag.insert_child), so they never land inside a cfRule's extLst.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019UZs6wsi5TT3GKqgC7bYeY
</commit_message>
<xml_diff>
--- a/examples/09-extensions.xlsx
+++ b/examples/09-extensions.xlsx
@@ -13,6 +13,28 @@
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -464,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -518,6 +540,16 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Sorted</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -546,6 +578,15 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="J2" cm="1">
+        <f t="array" ref="J2:J5">_xlfn._xlws.SORT(A2:A5)</f>
+        <v/>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0042</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -574,6 +615,11 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -602,6 +648,11 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -628,6 +679,11 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>Open</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>West</t>
         </is>
       </c>
     </row>
@@ -647,6 +703,9 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ignoredErrors>
+    <ignoredError sqref="K2" numberStoredAsText="1"/>
+  </ignoredErrors>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">

</xml_diff>